<commit_message>
added data and output files
</commit_message>
<xml_diff>
--- a/data/RuleFile.xlsx
+++ b/data/RuleFile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AgenticAIExcel\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C6CB1B-42F8-492B-BD82-3F2225E2220F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42757A88-9B89-4781-A9B5-0009B0DE7CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -469,20 +469,26 @@
     <t>Price, Nominal,Brokerage</t>
   </si>
   <si>
-    <t>Multiply price and nominal and divide result by brokerage and round to 4 decimal places</t>
+    <t>multiply price and nominal and divide result by brokerage</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF737780"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -505,8 +511,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -809,15 +818,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.3984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="69" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.53125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -828,7 +837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -839,7 +848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -850,7 +859,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -861,7 +870,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -872,7 +881,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -883,7 +892,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -894,7 +903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -905,7 +914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -915,8 +924,9 @@
       <c r="C9" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -927,7 +937,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -938,7 +948,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -949,7 +959,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -960,7 +970,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -971,7 +981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -982,7 +992,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -1842,5 +1852,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>